<commit_message>
test: regenerate V3 evaluation sample data
</commit_message>
<xml_diff>
--- a/public/test-data/01_과제_테스트.xlsx
+++ b/public/test-data/01_과제_테스트.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="과제양식" sheetId="1" r:id="R9576a00215e14e79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="과제양식" sheetId="1" r:id="Ra9b5b3884c8d4bee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="4">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -21,22 +21,16 @@
     <x:font>
       <x:b/>
       <x:sz val="10"/>
-      <x:color rgb="FFFFFFFF"/>
-      <x:name val="Arial"/>
+      <x:color rgb="FF111827"/>
+      <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF111827"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FF111827"/>
-      <x:name val="Arial"/>
+      <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -45,7 +39,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF111827"/>
+        <x:fgColor rgb="FFF3F4F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -69,7 +68,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="13">
+  <x:cellXfs count="14">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -83,19 +82,20 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -299,15 +299,15 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="11" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="9" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="24.440000534057617" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="8.329999923706055" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="32.220001220703125" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="33.33000183105469" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="28" customHeight="1">
+    <x:row r="1" ht="21" customHeight="1">
       <x:c r="A1" s="6" t="str">
         <x:v>과제명</x:v>
       </x:c>
@@ -327,63 +327,63 @@
         <x:v>성과등급</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="25" customHeight="1">
-      <x:c r="A2" s="11" t="str">
+    <x:row r="2" ht="21" customHeight="1">
+      <x:c r="A2" s="12" t="str">
         <x:v>신규 랜딩페이지 제작</x:v>
       </x:c>
-      <x:c r="B2" s="12" t="str">
+      <x:c r="B2" s="13" t="str">
         <x:v>핵심</x:v>
       </x:c>
-      <x:c r="C2" s="12" t="str">
+      <x:c r="C2" s="13" t="str">
         <x:v>대</x:v>
       </x:c>
       <x:c r="D2" s="12" t="str">
-        <x:v>전환율 15% 개선 및 모바일 이탈률 감소</x:v>
+        <x:v>전환율 15% 개선 및 신규 고객 유입 확대</x:v>
       </x:c>
       <x:c r="E2" s="12" t="str">
-        <x:v>전환율 18% 달성, 모바일 이탈률 12% 감소</x:v>
-      </x:c>
-      <x:c r="F2" s="12" t="str">
+        <x:v>전환율 18.6% 개선, 신규 유입 12.4% 증가</x:v>
+      </x:c>
+      <x:c r="F2" s="13" t="str">
         <x:v>A</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="25" customHeight="1">
-      <x:c r="A3" s="11" t="str">
+    <x:row r="3" ht="21" customHeight="1">
+      <x:c r="A3" s="12" t="str">
         <x:v>Cloud X 메인 UX 개선</x:v>
       </x:c>
-      <x:c r="B3" s="12" t="str">
+      <x:c r="B3" s="13" t="str">
         <x:v>중점</x:v>
       </x:c>
-      <x:c r="C3" s="12" t="str">
+      <x:c r="C3" s="13" t="str">
         <x:v>중</x:v>
       </x:c>
       <x:c r="D3" s="12" t="str">
-        <x:v>핵심 플로우 이탈률 20% 감소</x:v>
+        <x:v>핵심 업무 완료 시간을 20% 단축</x:v>
       </x:c>
       <x:c r="E3" s="12" t="str">
-        <x:v>이탈률 24% 감소, 주요 화면 사용성 개선 완료</x:v>
-      </x:c>
-      <x:c r="F3" s="12" t="str">
+        <x:v>완료 시간 24% 단축, 만족도 4.4점 달성</x:v>
+      </x:c>
+      <x:c r="F3" s="13" t="str">
         <x:v>S</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="25" customHeight="1">
-      <x:c r="A4" s="11" t="str">
+    <x:row r="4" ht="21" customHeight="1">
+      <x:c r="A4" s="12" t="str">
         <x:v>내부 협업툴 정비</x:v>
       </x:c>
-      <x:c r="B4" s="12" t="str">
+      <x:c r="B4" s="13" t="str">
         <x:v>일반</x:v>
       </x:c>
-      <x:c r="C4" s="12" t="str">
+      <x:c r="C4" s="13" t="str">
         <x:v>소</x:v>
       </x:c>
       <x:c r="D4" s="12" t="str">
-        <x:v>반복 업무 시간 10% 단축</x:v>
+        <x:v>중복 요청 30% 감소 및 업무 흐름 표준화</x:v>
       </x:c>
       <x:c r="E4" s="12" t="str">
-        <x:v>반복 업무 시간 12% 단축, 사용 가이드 배포</x:v>
-      </x:c>
-      <x:c r="F4" s="12" t="str">
+        <x:v>중복 요청 27% 감소, 표준 템플릿 8종 배포</x:v>
+      </x:c>
+      <x:c r="F4" s="13" t="str">
         <x:v>B</x:v>
       </x:c>
     </x:row>

</xml_diff>